<commit_message>
Refine loop semantics and validation pipeline
Clean up loop/candidate JSON, improve nested/sequential loop semantics, update Horn rule naming and validator generation, and refine experiment recording.
</commit_message>
<xml_diff>
--- a/experiment_results-old.xlsx
+++ b/experiment_results-old.xlsx
@@ -13,7 +13,7 @@
     <workbookView xWindow="2780" yWindow="1560" windowWidth="28040" windowHeight="17440" xr2:uid="{FF49B81A-127A-B44C-A44B-FF0F3EF8FCF9}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="gpt-5.6-terra" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -77,46 +77,40 @@
     <t>Initial Synthesis Cost (USD)</t>
   </si>
   <si>
-    <t>Grammar Refinement Calls</t>
-  </si>
-  <si>
-    <t>Grammar Refinement Time (ms)</t>
-  </si>
-  <si>
-    <t>Grammar Refinement Input Tokens</t>
-  </si>
-  <si>
-    <t>Grammar Refinement Output Tokens</t>
-  </si>
-  <si>
-    <t>Grammar Refinement Cost (USD)</t>
-  </si>
-  <si>
-    <t>Analysis Refinement Calls</t>
-  </si>
-  <si>
-    <t>Analysis Refinement Time (ms)</t>
-  </si>
-  <si>
-    <t>Analysis Refinement Input Tokens</t>
-  </si>
-  <si>
-    <t>Analysis Refinement Output Tokens</t>
-  </si>
-  <si>
-    <t>Analysis Refinement Cost (USD)</t>
+    <t>Syntactic Refinement Calls</t>
+  </si>
+  <si>
+    <t>Syntactic Refinement Time (ms)</t>
+  </si>
+  <si>
+    <t>Syntactic Refinement Input Tokens</t>
+  </si>
+  <si>
+    <t>Syntactic Refinement Output Tokens</t>
+  </si>
+  <si>
+    <t>Syntactic Refinement Cost (USD)</t>
+  </si>
+  <si>
+    <t>Semantic Refinement Calls</t>
+  </si>
+  <si>
+    <t>Semantic Refinement Time (ms)</t>
+  </si>
+  <si>
+    <t>Semantic Refinement Input Tokens</t>
+  </si>
+  <si>
+    <t>Semantic Refinement Output Tokens</t>
+  </si>
+  <si>
+    <t>Semantic Refinement Cost (USD)</t>
   </si>
   <si>
     <t>/Users/nfathi2/Documents/liveness_analysis/Nexus/artifacts/SourceCode.c</t>
   </si>
   <si>
     <t>non-terminating</t>
-  </si>
-  <si>
-    <t>terminating</t>
-  </si>
-  <si>
-    <t>error</t>
   </si>
 </sst>
 </file>
@@ -551,34 +545,34 @@
         <v>3</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G2">
-        <v>196</v>
+        <v>13147</v>
       </c>
       <c r="H2">
-        <v>201</v>
+        <v>13576</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>12976</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>22765</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>640</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>0.053209999999999993</v>
       </c>
       <c r="N2">
         <v>0</v>

</xml_diff>

<commit_message>
Improve refinement feedback history
Append per-loop syntactic and semantic feedback, include candidate context, and evaluate only the latest validator result.
</commit_message>
<xml_diff>
--- a/experiment_results-old.xlsx
+++ b/experiment_results-old.xlsx
@@ -554,25 +554,25 @@
         <v>25</v>
       </c>
       <c r="G2">
-        <v>13147</v>
+        <v>17371</v>
       </c>
       <c r="H2">
-        <v>13576</v>
+        <v>17814</v>
       </c>
       <c r="I2">
         <v>2</v>
       </c>
       <c r="J2">
-        <v>12976</v>
+        <v>17184</v>
       </c>
       <c r="K2">
         <v>22765</v>
       </c>
       <c r="L2">
-        <v>640</v>
+        <v>794</v>
       </c>
       <c r="M2">
-        <v>0.053209999999999993</v>
+        <v>0.014091800000000002</v>
       </c>
       <c r="N2">
         <v>0</v>

</xml_diff>